<commit_message>
Correction du scraper et ajout des resultats
</commit_message>
<xml_diff>
--- a/output_amazon_technologies/Ordinateurs portables/Ordinateurs portables.xlsx
+++ b/output_amazon_technologies/Ordinateurs portables/Ordinateurs portables.xlsx
@@ -540,34 +540,34 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://www.amazon.fr/dp/B0FHB6N6PP</t>
+          <t>https://www.amazon.fr/dp/B0HBWY6K1H</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>B0FHB6N6PP</t>
+          <t>B0HBWY6K1H</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Lenovo Chromebook Plus IdeaPad Slim 3 14IAN8 avec Google AI - Ordinateur Portable 14'' FHD (Intel Core i3-N305, RAM 8 Go, eMMC 128Go, ChromeOS) - Clavier AZERTY FR - Gris</t>
+          <t>Lenovo IdeaPad Slim 3 | Laptop | R7 | 16Go | 512Go | Chargeur Non Inclus</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>289,99€</t>
+          <t>699,99€</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Le Lenovo Chromebook Plus IdeaPad Slim 3 14IAN8 est un ordinateur portable moderne et performant, conçu pour offrir une expérience fluide sous ChromeOS. Équipé d’un écran 14 pouces Full HD, il propose un affichage net, idéal pour le travail, les cours en ligne ou les loisirs. Son processeur Intel Core i3-N305, associé à 8 Go de RAM et 128 Go de stockage eMMC, assure rapidité et efficacité au quotidien. Léger et facilement transportable, il dispose d’un clavier AZERTY français et d’une finition grise élégante. C’est le compagnon parfait pour les étudiants, les professionnels nomades ou toute personne à la recherche d’un Chromebook puissant, simple d’utilisation et fiable.</t>
+          <t>Le Lenovo IdeaPad Slim 3 15ABR8 est un ordinateur portable polyvalent conçu pour les tâches quotidiennes telles que la navigation sur Internet, le traitement de texte et la consommation de contenu multimédia. Il est équipé d'un processeur AMD Ryzen 7 5825U à 8 cœurs, offrant une fréquence de base de 4.0 GHz et pouvant atteindre 4.5 GHz en mode turbo, associé à 16 Go de RAM et un SSD de 512 Go pour un stockage rapide et spacieux. Son écran 15,6 pouces Full HD (1920 × 1080) avec technologie IPS et une luminosité de 300 nits assure une expérience visuelle claire et nette. De plus, il dispose de Wi-Fi 6, de ports USB-C, d'une caméra HD avec obturateur de confidentialité et d'une batterie de 47 Wh offrant une autonomie prolongée. Son design élégant et sa construction légère en font un choix idéal pour les étudiants et les professionnels en déplacement.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Les Chromebooks fonctionnent avec ChromeOS, le système d'exploitation rapide et sécurisé de Google. Cet appareil est conçu pour fonctionner avec ce système d'exploitation afin d'en optimiser les performances et la sécurité. [Connectez-vous simplement avec votre compte Google pour accéder instantanément aux applications Google Workspace intégrées, comme Docs et Sheets.]; Pour utiliser Microsoft 365, il vous suffit de vous rendre sur Microsoft365.com dans votre navigateur afin de créer et de modifier des documents Word, Excel et PowerPoint en ligne. Bien que les versions desktop ne soient pas installables, cette méthode offre un accès complet. Notez qu'un abonnement à Microsoft 365 est nécessaire pour accéder aux fonctionnalités supplémentaires.; LA MAGIE AU QUOTIDIEN AVEC GOOGLE AI: intègre de nouvelles fonctionnalités d’IA pour simplifier votre quotidien Discutez avec Gemini pour donner vie à vos idées, écrivez comme un pro ou encore retouchez vos photos en un clin d'œil grâce à l'IA de Google; PLUS DE PUISSANCE POUR PLUS D'EFFICACITÉ : profitez d'un processeur 2 fois plus rapide et jusqu’à 2 fois plus de RAM et de stockage pour modifier vos documents, photos et vidéos tout en regardant vos séries préférées sur un écran Full HD IPS; L'UTILISER C'EST L'ADOPTER : retrouvez les avantages du système d’exploitation ChromeOS, les Chromebooks n’ont jamais eu de virus Et avec jusqu'à 10h d'autonomie, un démarrage rapide et des mises à jour automatiques en arrière-plan, Chromebook Plus est aussi facile à utiliser qu’à aimer</t>
+          <t>Le chargeur n'est pas inclus avec ce modèle. Nous conseillons d'utiliser un chargeur Lenovo GaN Nano 65W .; Le Lenovo IdeaPad Slim 3 15ABR88 est doté d’un grand écran 15.6 pouces FHD pour une immersion visuelle optimale, idéale pour le travail multitâche et les contenus multimédias.; Le processeur AMD Ryzen 7 5825U offre une puissance exceptionnelle pour les tâches exigeantes comme la création de contenu, le montage ou les applications professionnelles.; Avec 16 Go de RAM et un SSD de 512 Go, cet ordinateur garantit une réactivité fluide et un espace de stockage rapide pour tous vos fichiers et projets.; Conçu avec un clavier AZERTY français et un design gris élégant, il allie confort, performance et esthétique pour un usage professionnel ou personnel intensif.</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -577,34 +577,34 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://www.amazon.fr/dp/B0HHGXHH3C</t>
+          <t>https://www.amazon.fr/dp/B0FHB6N6PP</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>B0HHGXHH3C</t>
+          <t>B0FHB6N6PP</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>18,5"Ordinateur Portable,Ryzen 7430U,16 Go DDR4 512 Go SSD,Usage Domestique</t>
+          <t>Lenovo Chromebook Plus IdeaPad Slim 3 14IAN8 avec Google AI - Ordinateur Portable 14'' FHD (Intel Core i3-N305, RAM 8 Go, eMMC 128Go, ChromeOS) - Clavier AZERTY FR - Gris</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>47,68 €</t>
+          <t>289,99€</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Description du produit 18,5" grand écran – ordinateur portable, idéal travail et films à la maison La vidéo présente le produit en cours d'utilisation. La vidéo vous guide tout au long de la configuration du produit. La vidéo compare plusieurs produits. La vidéo montre le produit en cours de déballage. Video Player is loading. Cliquez pour lire la vidéo Jouez Muet Current Time / Duration Loaded : 0% Stream Type LIVE Seek to live, currently behind live LIVE Remaining Time - 1x Playback Rate Chapters Chapters Descriptions descriptions off , selected Sous-titres Sous-titres désactivés , selected Audio Track default , selected Plein écran This is a modal window. 18,5"Ordinateur Portable,Ryzen 7430U Previous page Next page Previous page Next page Previous page Next page Previous page Next page Sélectionner ACEMAGIC, Sélectionner Laptop professionnel AX18PRO Options d’achat S16 Options d’achat LX15PRO Options d’achat AX17PRO Options d’achat AX18PRO Options d’achat Avis client 4,8 sur 5 étoiles 10 4,3 sur 5 étoiles 78 5,0 sur 5 étoiles 4 4,4 sur 5 étoiles 35 4,0 sur 5 étoiles 171 Usages du produit Usage domestique/Bureau Développeur Création multimédia/Affaires Étudiant/Divertissement Usage domestique/Étudiant Taille de l'écran 18,5 Pouces 16 Pouces 15,6 Pouces 17,3 Pouces 18,5 Pouces Modèle de processeur AMD Ryzen5 7430U AMD Ryzen7 H255 AMD Ryzen7 5825U AMD Ryzen3 4300U AMD Ryzen3 4300U Mémoire RAM 16Go 24Go 16Go 16Go 16Go Capacité de stockage 512Go 512Go 1000Go 512Go 512Go</t>
+          <t>Le Lenovo Chromebook Plus IdeaPad Slim 3 14IAN8 est un ordinateur portable moderne et performant, conçu pour offrir une expérience fluide sous ChromeOS. Équipé d’un écran 14 pouces Full HD, il propose un affichage net, idéal pour le travail, les cours en ligne ou les loisirs. Son processeur Intel Core i3-N305, associé à 8 Go de RAM et 128 Go de stockage eMMC, assure rapidité et efficacité au quotidien. Léger et facilement transportable, il dispose d’un clavier AZERTY français et d’une finition grise élégante. C’est le compagnon parfait pour les étudiants, les professionnels nomades ou toute personne à la recherche d’un Chromebook puissant, simple d’utilisation et fiable.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Grand écran de 18,5 pouces : Comparé à un écran de 15,6 pouces, l’écran de 18,5 pouces offre un champ visuel 36 % plus grand. Les caractères et icônes sont plus grands, pour un confort visuel accru. Il dispose d’une résolution Full HD 1920×1080 et d’un taux de rafraîchissement stable de 60 Hz, garantissant des images nettes et fluides. Grâce à sa charnière 180°, ajustez facilement l’angle sur canapé ou sur toutes les tables de la maison.; Processeur Ryzen 5 7430U : Cet ordinateur portable sous Win 11 Pro intègre le processeur Ryzen 5 7430U, doté de 6 cœurs et 12 threads, fréquence maximale pouvant atteindre 4,3 GHz. Carte graphique intégrée Radeon RX Vega 7, parfaitement adaptée au travail à domicile et à l'édition vidéo. Il bénéficie d’une grande mémoire cache L3 de 16 Mo pour une réactivité plus rapide des logiciels. L'ordinateur portable est préinstallé avec un système d'exploitation, prêt à l'usage dès le démarrage.; 16 Go DDR4 &amp; 512 Go SSD M.2 NVMe : L’ordinateur portable dispose de 16 Go de mémoire RAM DDR4 à 2666 MHz avec deux emplacements SO‑DIMM, extensible jusqu’à 64 Go. Le système reste fluide même lorsque de nombreuses pages web ou documents sont ouverts simultanément. Il intègre un SSD rapide M.2 NVMe PCIe3.0 de 512 Go, la capacité totale maximale de l’appareil peut atteindre 4 To ; vous pouvez conserver facilement de nombreuses photos de réunions familiales ou des vidéos de voyages.; WiFi 6 &amp; ports polyvalents : Équipé du WiFi 6 et du Bluetooth 5.2, la transmission des données est plus rapide. L’ordinateur portable dispose de nombreux ports : 2 × USB3.2, 1 × USB2.0, 2 × Type‑C, 1 × HDMI1.4, 1 × prise casque 3,5 mm et 1 × lecteur de carte TF. Satisfait facilement les besoins des appareils externes, idéal pour regarder des films en famille et projeter sur de grands écrans. Il est doté d’une webcam avec cache de confidentialité pour mieux protéger votre vie privée familiale.; Emballage &amp; support technique complet : Cet ordinateur portable Win 11 Pro est fourni avec de nombreux accessoires : 1 chargeur, 4 protections de clavier multilingues (espagnol, français, italien et allemand) et 1 manuel d’utilisation multilingue. L’ordinateur portable ACEMAGIC bénéficie d’une garantie de 24 mois et d’un support technique complet. Si vous avez des questions, n’hésitez pas à nous contacter à tout moment.</t>
+          <t>Les Chromebooks fonctionnent avec ChromeOS, le système d'exploitation rapide et sécurisé de Google. Cet appareil est conçu pour fonctionner avec ce système d'exploitation afin d'en optimiser les performances et la sécurité. [Connectez-vous simplement avec votre compte Google pour accéder instantanément aux applications Google Workspace intégrées, comme Docs et Sheets.]; Pour utiliser Microsoft 365, il vous suffit de vous rendre sur Microsoft365.com dans votre navigateur afin de créer et de modifier des documents Word, Excel et PowerPoint en ligne. Bien que les versions desktop ne soient pas installables, cette méthode offre un accès complet. Notez qu'un abonnement à Microsoft 365 est nécessaire pour accéder aux fonctionnalités supplémentaires.; LA MAGIE AU QUOTIDIEN AVEC GOOGLE AI: intègre de nouvelles fonctionnalités d’IA pour simplifier votre quotidien Discutez avec Gemini pour donner vie à vos idées, écrivez comme un pro ou encore retouchez vos photos en un clin d'œil grâce à l'IA de Google; PLUS DE PUISSANCE POUR PLUS D'EFFICACITÉ : profitez d'un processeur 2 fois plus rapide et jusqu’à 2 fois plus de RAM et de stockage pour modifier vos documents, photos et vidéos tout en regardant vos séries préférées sur un écran Full HD IPS; L'UTILISER C'EST L'ADOPTER : retrouvez les avantages du système d’exploitation ChromeOS, les Chromebooks n’ont jamais eu de virus Et avec jusqu'à 10h d'autonomie, un démarrage rapide et des mises à jour automatiques en arrière-plan, Chromebook Plus est aussi facile à utiliser qu’à aimer</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -614,34 +614,34 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://www.amazon.fr/dp/B0HBWY6K1H</t>
+          <t>https://www.amazon.fr/dp/B09BF96NHJ</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>B0HBWY6K1H</t>
+          <t>B09BF96NHJ</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Lenovo IdeaPad Slim 3 | Laptop | R7 | 16Go | 512Go | Chargeur Non Inclus</t>
+          <t>ASUS Vivobook 17 17.3 Pouces FHD PC Portable (Intel Core 7 150U, 16GB DDR5, 512GB SSD, Intel Graphics, Windows 11 Home) – Clavier AZERTY - sans Chargeur</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>699,99€</t>
+          <t>749,99€</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Le Lenovo IdeaPad Slim 3 15ABR8 est un ordinateur portable polyvalent conçu pour les tâches quotidiennes telles que la navigation sur Internet, le traitement de texte et la consommation de contenu multimédia. Il est équipé d'un processeur AMD Ryzen 7 5825U à 8 cœurs, offrant une fréquence de base de 4.0 GHz et pouvant atteindre 4.5 GHz en mode turbo, associé à 16 Go de RAM et un SSD de 512 Go pour un stockage rapide et spacieux. Son écran 15,6 pouces Full HD (1920 × 1080) avec technologie IPS et une luminosité de 300 nits assure une expérience visuelle claire et nette. De plus, il dispose de Wi-Fi 6, de ports USB-C, d'une caméra HD avec obturateur de confidentialité et d'une batterie de 47 Wh offrant une autonomie prolongée. Son design élégant et sa construction légère en font un choix idéal pour les étudiants et les professionnels en déplacement.</t>
+          <t>Le ASUS Vivobook 17 X1704VA-AU1185W est un ordinateur portable polyvalent conçu pour répondre à vos besoins quotidiens en matière de travail, de divertissement et de communication. Son grand écran FHD de 17,3 pouces offre une expérience visuelle confortable, tandis que le processeur Intel Core 7 150U et la mémoire DDR5 de 16GB assurent une performance polyvalente pour la plupart des tâches courantes. Le stockage SSD de 512GB M.2 NVMe PCIe 4.0 offre des temps de démarrage rapides et des chargements d'applications quasi instantanés. La connectivité complète, avec Wi-Fi 6 et Bluetooth 5.2, vous permet de rester connecté où que vous soyez. Les ports E/S incluent 1x USB 2.0 Type-A, 1x USB 3.2 Gen 1 Type-C, 1x USB 3.2 Gen 1 Type-C avec support Power Delivery, 2x USB 3.2 Gen 1 Type-A et 1x HDMI 1.4, vous offrant une connectivité complète pour tous vos périphériques. Le design robuste et fiable du ASUS Vivobook 17 X1704VA-AU1185W répond à la norme militaire US MIL-STD 810H, assurant une durabilité exceptionnelle. L'expérience audio claire, avec la technologie SonicMaster, vous permet de profiter d'un son clair pour tous vos contenus. La sécurité et la confidentialité sont renforcées par la caméra HD 720p avec obturateur de confidentialité et le module TPM (Firmware TPM). Les logiciels utiles préinstallés, tels que MyASUS, ScreenXpert et GlideX, vous offrent des fonctionnalités supplémentaires pour optimiser votre expérience utilisateur. En résumé, le ASUS Vivobook 17 X1704VA-AU1185W est un excellent choix pour ceux qui recherchent un ordinateur portable fiable, performant et abordable avec un grand écran pour toutes leurs tâches quotidiennes.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Le chargeur n'est pas inclus avec ce modèle. Nous conseillons d'utiliser un chargeur Lenovo GaN Nano 65W .; Le Lenovo IdeaPad Slim 3 15ABR88 est doté d’un grand écran 15.6 pouces FHD pour une immersion visuelle optimale, idéale pour le travail multitâche et les contenus multimédias.; Le processeur AMD Ryzen 7 5825U offre une puissance exceptionnelle pour les tâches exigeantes comme la création de contenu, le montage ou les applications professionnelles.; Avec 16 Go de RAM et un SSD de 512 Go, cet ordinateur garantit une réactivité fluide et un espace de stockage rapide pour tous vos fichiers et projets.; Conçu avec un clavier AZERTY français et un design gris élégant, il allie confort, performance et esthétique pour un usage professionnel ou personnel intensif.</t>
+          <t>Conception Robuste et Fiable : Le ASUS Vivobook 17 X1704VA-AU1185W est conçu pour résister aux rigueurs de la vie quotidienne. Il répond à la norme militaire US MIL-STD 810H, assurant une durabilité exceptionnelle. Son design élégant en Cool Silver lui confère un aspect sobre et professionnel. Avec un poids de seulement 2,10 kg, il reste relativement facile à transporter pour un ordinateur portable de cette taille.</t>
         </is>
       </c>
       <c r="I6" t="n">

</xml_diff>